<commit_message>
Fixed studies tab anatomic-site queries
</commit_message>
<xml_diff>
--- a/InputFiles/C3DC/TC01_C3DC_phs000463_SexAtBirth-Female.xlsx
+++ b/InputFiles/C3DC/TC01_C3DC_phs000463_SexAtBirth-Female.xlsx
@@ -584,11 +584,20 @@
      diagnosis_all[0..5] AS diagnosis_items,
      size(diagnosis_all) &gt; 5 AS diagnosis_more
 OPTIONAL MATCH (d2:diagnosis)-[:of_diagnosis]-&gt;(dp2:participant)-[:of_participant]-&gt;(:consent_group)-[:of_consent_group]-&gt;(s)
-UNWIND CASE WHEN d2 IS NULL THEN [null] ELSE coalesce(d2.anatomic_site, [null]) END AS site
+UNWIND CASE
+  WHEN d2 IS NULL THEN []
+  WHEN size(coalesce(d2.anatomic_site, [])) = 0 THEN [null]
+  ELSE d2.anatomic_site
+END AS site_raw
+WITH s, num_of_participants, num_of_samples, diagnosis_items, diagnosis_more, d2, site_raw,
+     CASE
+       WHEN site_raw IS NULL OR trim(toString(site_raw)) = '' THEN 'Not Reported'
+       ELSE site_raw
+     END AS site
 WITH s, num_of_participants, num_of_samples, diagnosis_items, diagnosis_more, site, count(DISTINCT d2) AS site_n
-ORDER BY site_n DESC, site DESC
+ORDER BY site_n DESC, site ASC
 WITH s, num_of_participants, num_of_samples, diagnosis_items, diagnosis_more,
-     [item IN collect(CASE WHEN site IS NULL THEN null ELSE site + ' (' + toString(site_n) + ')' END) WHERE item IS NOT NULL] AS site_all
+     collect(site + ' (' + toString(site_n) + ')') AS site_all
 WITH s, num_of_participants, num_of_samples, diagnosis_items, diagnosis_more,
      site_all[0..5] AS site_items,
      size(site_all) &gt; 5 AS site_more

</xml_diff>